<commit_message>
Sinyi links via sinyiglobal; Zhongding list photos
</commit_message>
<xml_diff>
--- a/office-analysis.xlsx
+++ b/office-analysis.xlsx
@@ -452,7 +452,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3539" uniqueCount="1233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3539" uniqueCount="1232">
   <si>
     <r>
       <rPr>
@@ -3373,7 +3373,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">信義國際站 本戶·14張照片（備用：www.sinyi.com.tw/rent/houseno/C355686）</t>
+    <t xml:space="preserve">信義全球 本戶·14張照片（C355686）</t>
   </si>
   <si>
     <t xml:space="preserve">Y1</t>
@@ -32150,7 +32150,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">https://www.sinyi.com.tw/rent/houseno/CZ05290</t>
+    <t xml:space="preserve">https://www.sinyiglobal.com/rental/CZ05290</t>
   </si>
   <si>
     <r>
@@ -34709,7 +34709,7 @@
     <t xml:space="preserve">白宮企業大樓 — 同層參考(非本案) ↗</t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.sinyi.com.tw/rent/houseno/C351775</t>
+    <t xml:space="preserve">https://www.sinyiglobal.com/rental/C351775</t>
   </si>
   <si>
     <r>
@@ -35630,7 +35630,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">https://www.sinyi.com.tw/rent/houseno/CZ05572</t>
+    <t xml:space="preserve">https://www.sinyiglobal.com/rental/CZ05572</t>
   </si>
   <si>
     <r>
@@ -35754,7 +35754,7 @@
     <t xml:space="preserve">中鼎大樓 2F ↗</t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.sinyi.com.tw/rent/houseno/CZ05228</t>
+    <t xml:space="preserve">https://www.sinyiglobal.com/rental/CZ05228</t>
   </si>
   <si>
     <r>
@@ -35847,7 +35847,7 @@
     <t xml:space="preserve">家美金融大樓 15F ↗</t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.sinyi.com.tw/rent/houseno/CZ05491</t>
+    <t xml:space="preserve">https://www.sinyiglobal.com/rental/CZ05491</t>
   </si>
   <si>
     <r>
@@ -36373,9 +36373,6 @@
       </rPr>
       <t xml:space="preserve">更新</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.sinyi.com.tw/rent/houseno/C355686</t>
   </si>
   <si>
     <t xml:space="preserve">信義房屋 主站</t>
@@ -46814,7 +46811,7 @@
     <hyperlink ref="B12" r:id="rId16" display="591 光復南路 7F ↗"/>
     <hyperlink ref="W12" r:id="rId17" display="HouseWeb 本戶·40張照片"/>
     <hyperlink ref="B13" r:id="rId18" display="信義 光復北路新大樓 5F ↗"/>
-    <hyperlink ref="W13" r:id="rId19" display="信義國際站 本戶·14張照片（備用：www.sinyi.com.tw/rent/houseno/C355686）"/>
+    <hyperlink ref="W13" r:id="rId19" display="信義全球 本戶·14張照片（C355686）"/>
     <hyperlink ref="B14" r:id="rId20" display="永慶 安敦國際大樓 14F ↗"/>
     <hyperlink ref="W14" r:id="rId21" display="永慶 本戶14F·15張照片"/>
     <hyperlink ref="B15" r:id="rId22" display="永慶／信義 家美金融大樓 15F ↗"/>
@@ -46843,7 +46840,7 @@
     <hyperlink ref="W26" r:id="rId45" display="信義 本戶·18張照片（C360351）"/>
     <hyperlink ref="B31" r:id="rId46" display="https://business.591.com.tw/rent/22034644"/>
     <hyperlink ref="O31" r:id="rId47" display="591 本戶7F·14張照片"/>
-    <hyperlink ref="B32" r:id="rId48" display="https://www.sinyi.com.tw/rent/houseno/CZ05572"/>
+    <hyperlink ref="B32" r:id="rId48" display="https://www.sinyiglobal.com/rental/CZ05572"/>
     <hyperlink ref="O32" r:id="rId49" display="信義 本戶15F·15張照片（CZ05572）"/>
     <hyperlink ref="B33" r:id="rId50" display="https://buy.housefun.com.tw/buy/building/9278"/>
     <hyperlink ref="O33" r:id="rId51" display="好房網大樓頁·19張照片(本戶無公開頁)"/>
@@ -46858,32 +46855,32 @@
     <hyperlink ref="B38" r:id="rId60" display="https://www.houseweb.com.tw/house/2653888"/>
     <hyperlink ref="O38" r:id="rId61" display="HouseWeb 本戶·40張照片"/>
     <hyperlink ref="B39" r:id="rId62" display="https://www.sinyiglobal.com/rental/C355686"/>
-    <hyperlink ref="O39" r:id="rId63" display="信義國際站 本戶·14張照片（備用：www.sinyi.com.tw/rent/houseno/C355686）"/>
+    <hyperlink ref="O39" r:id="rId63" display="信義全球 本戶·14張照片（C355686）"/>
     <hyperlink ref="B40" r:id="rId64" display="https://rent.yungching.com.tw/region/house/2358272?pc=0916263633"/>
     <hyperlink ref="O40" r:id="rId65" display="永慶 本戶14F·15張照片"/>
     <hyperlink ref="B41" r:id="rId66" display="https://rent.yungching.com.tw/region/house/2373308?pc=0916263633"/>
     <hyperlink ref="O41" r:id="rId67" display="永慶 本戶15F·14張照片"/>
-    <hyperlink ref="B42" r:id="rId68" display="https://www.sinyi.com.tw/rent/houseno/CZ05326"/>
+    <hyperlink ref="B42" r:id="rId68" display="https://www.sinyiglobal.com/rental/CZ05326"/>
     <hyperlink ref="O42" r:id="rId69" display="信義 本戶·21張照片（CZ05326）"/>
-    <hyperlink ref="B43" r:id="rId70" display="https://www.sinyi.com.tw/rent/houseno/C328671"/>
+    <hyperlink ref="B43" r:id="rId70" display="https://www.sinyiglobal.com/rental/C328671"/>
     <hyperlink ref="O43" r:id="rId71" display="信義 本戶·19張照片（C328671）"/>
-    <hyperlink ref="B44" r:id="rId72" display="https://www.sinyi.com.tw/rent/houseno/C905199"/>
+    <hyperlink ref="B44" r:id="rId72" display="https://www.sinyiglobal.com/rental/C905199"/>
     <hyperlink ref="O44" r:id="rId73" display="信義 本戶·16張照片（C905199）"/>
-    <hyperlink ref="B45" r:id="rId74" display="https://www.sinyi.com.tw/rent/houseno/CZ05587"/>
+    <hyperlink ref="B45" r:id="rId74" display="https://www.sinyiglobal.com/rental/CZ05587"/>
     <hyperlink ref="O45" r:id="rId75" display="信義 本戶·9張照片（CZ05587）"/>
-    <hyperlink ref="B46" r:id="rId76" display="https://www.sinyi.com.tw/rent/houseno/CZ03701"/>
+    <hyperlink ref="B46" r:id="rId76" display="https://www.sinyiglobal.com/rental/CZ03701"/>
     <hyperlink ref="O46" r:id="rId77" display="信義 本戶·12張照片（CZ03701）"/>
-    <hyperlink ref="B47" r:id="rId78" display="https://www.sinyi.com.tw/rent/houseno/C346398"/>
+    <hyperlink ref="B47" r:id="rId78" display="https://www.sinyiglobal.com/rental/C346398"/>
     <hyperlink ref="O47" r:id="rId79" display="信義 本戶·12張照片（C346398）"/>
-    <hyperlink ref="B48" r:id="rId80" display="https://www.sinyi.com.tw/rent/houseno/CZ05585"/>
+    <hyperlink ref="B48" r:id="rId80" display="https://www.sinyiglobal.com/rental/CZ05585"/>
     <hyperlink ref="O48" r:id="rId81" display="信義 本戶（CZ05585）"/>
-    <hyperlink ref="B49" r:id="rId82" display="https://www.sinyi.com.tw/rent/houseno/C904707"/>
+    <hyperlink ref="B49" r:id="rId82" display="https://www.sinyiglobal.com/rental/C904707"/>
     <hyperlink ref="O49" r:id="rId83" display="信義 本戶（C904707）"/>
-    <hyperlink ref="B50" r:id="rId84" display="https://www.sinyi.com.tw/rent/houseno/C360646"/>
+    <hyperlink ref="B50" r:id="rId84" display="https://www.sinyiglobal.com/rental/C360646"/>
     <hyperlink ref="O50" r:id="rId85" display="信義 本戶（C360646）"/>
-    <hyperlink ref="B51" r:id="rId86" display="https://www.sinyi.com.tw/rent/houseno/C348029"/>
+    <hyperlink ref="B51" r:id="rId86" display="https://www.sinyiglobal.com/rental/C348029"/>
     <hyperlink ref="O51" r:id="rId87" display="信義 本戶·5張照片（C348029）"/>
-    <hyperlink ref="B52" r:id="rId88" display="https://www.sinyi.com.tw/rent/houseno/C360351"/>
+    <hyperlink ref="B52" r:id="rId88" display="https://www.sinyiglobal.com/rental/C360351"/>
     <hyperlink ref="O52" r:id="rId89" display="信義 本戶·18張照片（C360351）"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -46912,132 +46909,132 @@
   <sheetData>
     <row r="1" customFormat="false" ht="20.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>1149</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="97" t="s">
+        <v>1150</v>
+      </c>
+      <c r="B4" s="98" t="s">
         <v>1151</v>
       </c>
-      <c r="B4" s="98" t="s">
+      <c r="C4" s="97" t="s">
         <v>1152</v>
-      </c>
-      <c r="C4" s="97" t="s">
-        <v>1153</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="39" t="s">
+        <v>1153</v>
+      </c>
+      <c r="B5" s="12" t="s">
         <v>1154</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="C5" s="39" t="s">
         <v>1155</v>
-      </c>
-      <c r="C5" s="39" t="s">
-        <v>1156</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="39" t="s">
+        <v>1156</v>
+      </c>
+      <c r="B6" s="12" t="s">
         <v>1157</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="C6" s="39" t="s">
         <v>1158</v>
-      </c>
-      <c r="C6" s="39" t="s">
-        <v>1159</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="39" t="s">
+        <v>1159</v>
+      </c>
+      <c r="B7" s="12" t="s">
         <v>1160</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="C7" s="39" t="s">
         <v>1161</v>
-      </c>
-      <c r="C7" s="39" t="s">
-        <v>1162</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="39" t="s">
+        <v>1162</v>
+      </c>
+      <c r="B8" s="12" t="s">
         <v>1163</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="C8" s="39" t="s">
         <v>1164</v>
-      </c>
-      <c r="C8" s="39" t="s">
-        <v>1165</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="39" t="s">
+        <v>1165</v>
+      </c>
+      <c r="B9" s="12" t="s">
         <v>1166</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="C9" s="39" t="s">
         <v>1167</v>
-      </c>
-      <c r="C9" s="39" t="s">
-        <v>1168</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="39" t="s">
+        <v>1168</v>
+      </c>
+      <c r="B10" s="12" t="s">
         <v>1169</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="C10" s="39" t="s">
         <v>1170</v>
-      </c>
-      <c r="C10" s="39" t="s">
-        <v>1171</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="43" t="s">
+        <v>1171</v>
+      </c>
+      <c r="B11" s="12" t="s">
         <v>1172</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="C11" s="39" t="s">
         <v>1173</v>
-      </c>
-      <c r="C11" s="39" t="s">
-        <v>1174</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="39" t="s">
+        <v>1174</v>
+      </c>
+      <c r="B12" s="7" t="s">
         <v>1175</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="C12" s="39" t="s">
         <v>1176</v>
-      </c>
-      <c r="C12" s="39" t="s">
-        <v>1177</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="39" t="s">
+        <v>1177</v>
+      </c>
+      <c r="B13" s="12" t="s">
         <v>1178</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="C13" s="39" t="s">
         <v>1179</v>
-      </c>
-      <c r="C13" s="39" t="s">
-        <v>1180</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="99" t="s">
-        <v>1182</v>
+        <v>1181</v>
       </c>
       <c r="B17" s="99"/>
       <c r="C17" s="99"/>
@@ -47101,12 +47098,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>1183</v>
+        <v>1182</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="97" t="s">
-        <v>1184</v>
+        <v>1183</v>
       </c>
       <c r="B3" s="97" t="s">
         <v>563</v>
@@ -47117,200 +47114,200 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="43" t="s">
+        <v>1184</v>
+      </c>
+      <c r="B4" s="39" t="s">
         <v>1185</v>
       </c>
-      <c r="B4" s="39" t="s">
+      <c r="C4" s="39" t="s">
         <v>1186</v>
-      </c>
-      <c r="C4" s="39" t="s">
-        <v>1187</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="43" t="s">
+        <v>1187</v>
+      </c>
+      <c r="B5" s="39" t="s">
         <v>1188</v>
       </c>
-      <c r="B5" s="39" t="s">
+      <c r="C5" s="39" t="s">
         <v>1189</v>
-      </c>
-      <c r="C5" s="39" t="s">
-        <v>1190</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="43" t="s">
+        <v>1190</v>
+      </c>
+      <c r="B6" s="39" t="s">
         <v>1191</v>
       </c>
-      <c r="B6" s="39" t="s">
-        <v>1192</v>
-      </c>
       <c r="C6" s="39" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="43" t="s">
+        <v>1192</v>
+      </c>
+      <c r="B7" s="39" t="s">
         <v>1193</v>
       </c>
-      <c r="B7" s="39" t="s">
-        <v>1194</v>
-      </c>
       <c r="C7" s="39" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="43" t="s">
+        <v>1194</v>
+      </c>
+      <c r="B8" s="39" t="s">
         <v>1195</v>
       </c>
-      <c r="B8" s="39" t="s">
-        <v>1196</v>
-      </c>
       <c r="C8" s="39" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="43" t="s">
+        <v>1196</v>
+      </c>
+      <c r="B9" s="39" t="s">
         <v>1197</v>
       </c>
-      <c r="B9" s="39" t="s">
-        <v>1198</v>
-      </c>
       <c r="C9" s="39" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="43" t="s">
+        <v>1198</v>
+      </c>
+      <c r="B10" s="39" t="s">
         <v>1199</v>
       </c>
-      <c r="B10" s="39" t="s">
-        <v>1200</v>
-      </c>
       <c r="C10" s="39" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="43" t="s">
-        <v>1201</v>
+        <v>1200</v>
       </c>
       <c r="B11" s="43" t="s">
         <v>983</v>
       </c>
       <c r="C11" s="39" t="s">
-        <v>1202</v>
+        <v>1201</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="43" t="s">
-        <v>1203</v>
+        <v>1202</v>
       </c>
       <c r="B12" s="43" t="s">
         <v>902</v>
       </c>
       <c r="C12" s="39" t="s">
-        <v>1202</v>
+        <v>1201</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="43" t="s">
+        <v>1203</v>
+      </c>
+      <c r="B13" s="39" t="s">
         <v>1204</v>
       </c>
-      <c r="B13" s="39" t="s">
+      <c r="C13" s="39" t="s">
         <v>1205</v>
-      </c>
-      <c r="C13" s="39" t="s">
-        <v>1206</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="43" t="s">
+        <v>1206</v>
+      </c>
+      <c r="B14" s="39" t="s">
         <v>1207</v>
       </c>
-      <c r="B14" s="39" t="s">
-        <v>1208</v>
-      </c>
       <c r="C14" s="39" t="s">
-        <v>1206</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="43" t="s">
+        <v>1208</v>
+      </c>
+      <c r="B15" s="39" t="s">
         <v>1209</v>
       </c>
-      <c r="B15" s="39" t="s">
-        <v>1210</v>
-      </c>
       <c r="C15" s="39" t="s">
-        <v>1206</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="39" t="s">
+        <v>1210</v>
+      </c>
+      <c r="B16" s="39" t="s">
         <v>1211</v>
       </c>
-      <c r="B16" s="39" t="s">
+      <c r="C16" s="39" t="s">
         <v>1212</v>
-      </c>
-      <c r="C16" s="39" t="s">
-        <v>1213</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="43" t="s">
+        <v>1213</v>
+      </c>
+      <c r="B17" s="43" t="s">
         <v>1214</v>
       </c>
-      <c r="B17" s="43" t="s">
+      <c r="C17" s="43" t="s">
         <v>1215</v>
-      </c>
-      <c r="C17" s="43" t="s">
-        <v>1216</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="43" t="s">
+        <v>1216</v>
+      </c>
+      <c r="B18" s="43" t="s">
+        <v>1013</v>
+      </c>
+      <c r="C18" s="39" t="s">
         <v>1217</v>
-      </c>
-      <c r="B18" s="43" t="s">
-        <v>1016</v>
-      </c>
-      <c r="C18" s="39" t="s">
-        <v>1218</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="43" t="s">
+        <v>1218</v>
+      </c>
+      <c r="B19" s="43" t="s">
         <v>1219</v>
       </c>
-      <c r="B19" s="43" t="s">
+      <c r="C19" s="39" t="s">
         <v>1220</v>
-      </c>
-      <c r="C19" s="39" t="s">
-        <v>1221</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="41" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="43" t="s">
+        <v>1221</v>
+      </c>
+      <c r="B20" s="43" t="s">
         <v>1222</v>
       </c>
-      <c r="B20" s="43" t="s">
+      <c r="C20" s="43" t="s">
         <v>1223</v>
-      </c>
-      <c r="C20" s="43" t="s">
-        <v>1224</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="43" t="s">
+        <v>1224</v>
+      </c>
+      <c r="B21" s="39" t="s">
         <v>1225</v>
       </c>
-      <c r="B21" s="39" t="s">
+      <c r="C21" s="39" t="s">
         <v>1226</v>
-      </c>
-      <c r="C21" s="39" t="s">
-        <v>1227</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -47318,21 +47315,21 @@
         <v>264</v>
       </c>
       <c r="B22" s="39" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C22" s="39" t="s">
         <v>1228</v>
-      </c>
-      <c r="C22" s="39" t="s">
-        <v>1229</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="39" t="s">
+        <v>1229</v>
+      </c>
+      <c r="B23" s="39" t="s">
         <v>1230</v>
       </c>
-      <c r="B23" s="39" t="s">
+      <c r="C23" s="43" t="s">
         <v>1231</v>
-      </c>
-      <c r="C23" s="43" t="s">
-        <v>1232</v>
       </c>
     </row>
   </sheetData>
@@ -52124,7 +52121,7 @@
     <hyperlink ref="D20" r:id="rId31" display="▲敦南商圈【氣派純辦】【裝潢新】 ↗"/>
     <hyperlink ref="AA20" r:id="rId32" display="HouseWeb·26張"/>
     <hyperlink ref="D21" r:id="rId33" display="信義 光復北路新大樓 5F ↗"/>
-    <hyperlink ref="AA21" r:id="rId34" display="信義國際站 本戶·14張照片（備用：www.sinyi.com.tw/rent/houseno/C355686）"/>
+    <hyperlink ref="AA21" r:id="rId34" display="信義全球 本戶·14張照片（C355686）"/>
     <hyperlink ref="D22" r:id="rId35" display="友聯大樓 5F ↗"/>
     <hyperlink ref="AA22" r:id="rId36" display="友聯5F 現況室內8張照片（591刊登圖·使用者提供）"/>
     <hyperlink ref="D23" r:id="rId37" location="page=1" display="信義路5段(環球) 18F 201坪 ↗"/>
@@ -56310,7 +56307,7 @@
     <hyperlink ref="D10" r:id="rId7" location="page=3" display="八德路vs龍江路 2F 220坪 ↗"/>
     <hyperlink ref="Z10" r:id="rId8" location="page=3" display="傑森愛華原始PDF 第3頁（此列無照片）"/>
     <hyperlink ref="D11" r:id="rId9" display="信義 光復北路新大樓 5F ↗"/>
-    <hyperlink ref="Z11" r:id="rId10" display="信義國際站 本戶·14張照片（備用：www.sinyi.com.tw/rent/houseno/C355686）"/>
+    <hyperlink ref="Z11" r:id="rId10" display="信義全球 本戶·14張照片（C355686）"/>
     <hyperlink ref="D12" r:id="rId11" display="信義 八德正核心大辦公室 7F ↗"/>
     <hyperlink ref="Z12" r:id="rId12" display="信義 本戶·9張照片（CZ05587）"/>
     <hyperlink ref="D13" r:id="rId13" location="page=1" display="信義路5段(環球) 18F 201坪 ↗"/>
@@ -56823,7 +56820,7 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C5" r:id="rId1" display="信義 光復北路新大樓 5F ↗"/>
-    <hyperlink ref="I5" r:id="rId2" display="信義國際站 本戶·14張照片（備用：www.sinyi.com.tw/rent/houseno/C355686）"/>
+    <hyperlink ref="I5" r:id="rId2" display="信義全球 本戶·14張照片（C355686）"/>
     <hyperlink ref="C6" r:id="rId3" display="中鼎大樓 15F / 2F / 22F ↗"/>
     <hyperlink ref="I6" r:id="rId4" display="信義 本戶15F·15張照片（CZ05572）"/>
     <hyperlink ref="C7" r:id="rId5" display="國泰世華銀行大樓 6F ↗"/>
@@ -60919,7 +60916,7 @@
   <hyperlinks>
     <hyperlink ref="C5" r:id="rId1" display="https://business.591.com.tw/rent/22034644"/>
     <hyperlink ref="J5" r:id="rId2" display="591 本戶7F·14張照片"/>
-    <hyperlink ref="C6" r:id="rId3" display="https://www.sinyi.com.tw/rent/houseno/CZ05572"/>
+    <hyperlink ref="C6" r:id="rId3" display="https://www.sinyiglobal.com/rental/CZ05572"/>
     <hyperlink ref="J6" r:id="rId4" display="信義 本戶15F·15張照片（CZ05572）"/>
     <hyperlink ref="C7" r:id="rId5" display="https://buy.housefun.com.tw/buy/building/9278"/>
     <hyperlink ref="J7" r:id="rId6" display="好房網大樓頁·19張照片(本戶無公開頁)"/>
@@ -60934,32 +60931,32 @@
     <hyperlink ref="C12" r:id="rId15" display="https://www.houseweb.com.tw/house/2653888"/>
     <hyperlink ref="J12" r:id="rId16" display="HouseWeb 本戶·40張照片"/>
     <hyperlink ref="C13" r:id="rId17" display="https://www.sinyiglobal.com/rental/C355686"/>
-    <hyperlink ref="J13" r:id="rId18" display="信義國際站 本戶·14張照片（備用：www.sinyi.com.tw/rent/houseno/C355686）"/>
+    <hyperlink ref="J13" r:id="rId18" display="信義全球 本戶·14張照片（C355686）"/>
     <hyperlink ref="C14" r:id="rId19" display="https://rent.yungching.com.tw/region/house/2358272?pc=0916263633"/>
     <hyperlink ref="J14" r:id="rId20" display="永慶 本戶14F·15張照片"/>
     <hyperlink ref="C15" r:id="rId21" display="https://rent.yungching.com.tw/region/house/2373308?pc=0916263633"/>
     <hyperlink ref="J15" r:id="rId22" display="永慶 本戶15F·14張照片"/>
-    <hyperlink ref="C16" r:id="rId23" display="https://www.sinyi.com.tw/rent/houseno/CZ05326"/>
+    <hyperlink ref="C16" r:id="rId23" display="https://www.sinyiglobal.com/rental/CZ05326"/>
     <hyperlink ref="J16" r:id="rId24" display="信義 本戶·21張照片（CZ05326）"/>
-    <hyperlink ref="C17" r:id="rId25" display="https://www.sinyi.com.tw/rent/houseno/C328671"/>
+    <hyperlink ref="C17" r:id="rId25" display="https://www.sinyiglobal.com/rental/C328671"/>
     <hyperlink ref="J17" r:id="rId26" display="信義 本戶·19張照片（C328671）"/>
-    <hyperlink ref="C18" r:id="rId27" display="https://www.sinyi.com.tw/rent/houseno/C905199"/>
+    <hyperlink ref="C18" r:id="rId27" display="https://www.sinyiglobal.com/rental/C905199"/>
     <hyperlink ref="J18" r:id="rId28" display="信義 本戶·16張照片（C905199）"/>
-    <hyperlink ref="C19" r:id="rId29" display="https://www.sinyi.com.tw/rent/houseno/CZ05587"/>
+    <hyperlink ref="C19" r:id="rId29" display="https://www.sinyiglobal.com/rental/CZ05587"/>
     <hyperlink ref="J19" r:id="rId30" display="信義 本戶·9張照片（CZ05587）"/>
-    <hyperlink ref="C20" r:id="rId31" display="https://www.sinyi.com.tw/rent/houseno/CZ03701"/>
+    <hyperlink ref="C20" r:id="rId31" display="https://www.sinyiglobal.com/rental/CZ03701"/>
     <hyperlink ref="J20" r:id="rId32" display="信義 本戶·12張照片（CZ03701）"/>
-    <hyperlink ref="C21" r:id="rId33" display="https://www.sinyi.com.tw/rent/houseno/C346398"/>
+    <hyperlink ref="C21" r:id="rId33" display="https://www.sinyiglobal.com/rental/C346398"/>
     <hyperlink ref="J21" r:id="rId34" display="信義 本戶·12張照片（C346398）"/>
-    <hyperlink ref="C22" r:id="rId35" display="https://www.sinyi.com.tw/rent/houseno/CZ05585"/>
+    <hyperlink ref="C22" r:id="rId35" display="https://www.sinyiglobal.com/rental/CZ05585"/>
     <hyperlink ref="J22" r:id="rId36" display="信義 本戶（CZ05585）"/>
-    <hyperlink ref="C23" r:id="rId37" display="https://www.sinyi.com.tw/rent/houseno/C904707"/>
+    <hyperlink ref="C23" r:id="rId37" display="https://www.sinyiglobal.com/rental/C904707"/>
     <hyperlink ref="J23" r:id="rId38" display="信義 本戶（C904707）"/>
-    <hyperlink ref="C24" r:id="rId39" display="https://www.sinyi.com.tw/rent/houseno/C360646"/>
+    <hyperlink ref="C24" r:id="rId39" display="https://www.sinyiglobal.com/rental/C360646"/>
     <hyperlink ref="J24" r:id="rId40" display="信義 本戶（C360646）"/>
-    <hyperlink ref="C25" r:id="rId41" display="https://www.sinyi.com.tw/rent/houseno/C348029"/>
+    <hyperlink ref="C25" r:id="rId41" display="https://www.sinyiglobal.com/rental/C348029"/>
     <hyperlink ref="J25" r:id="rId42" display="信義 本戶·5張照片（C348029）"/>
-    <hyperlink ref="C26" r:id="rId43" display="https://www.sinyi.com.tw/rent/houseno/C360351"/>
+    <hyperlink ref="C26" r:id="rId43" display="https://www.sinyiglobal.com/rental/C360351"/>
     <hyperlink ref="J26" r:id="rId44" display="信義 本戶·18張照片（C360351）"/>
     <hyperlink ref="C27" r:id="rId45" display="https://www.houseweb.com.tw/house/1506073"/>
     <hyperlink ref="J27" r:id="rId46" display="HouseWeb·26張"/>
@@ -61936,16 +61933,16 @@
         <v>106</v>
       </c>
       <c r="C42" s="13" t="s">
+        <v>1013</v>
+      </c>
+      <c r="D42" s="63" t="s">
         <v>1016</v>
       </c>
-      <c r="D42" s="63" t="s">
+      <c r="E42" s="63" t="s">
         <v>1017</v>
       </c>
-      <c r="E42" s="63" t="s">
+      <c r="F42" s="63" t="s">
         <v>1018</v>
-      </c>
-      <c r="F42" s="63" t="s">
-        <v>1019</v>
       </c>
       <c r="G42" s="38" t="s">
         <v>367</v>
@@ -61959,7 +61956,7 @@
         <v>793</v>
       </c>
       <c r="C43" s="13" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
       <c r="D43" s="63" t="s">
         <v>924</v>
@@ -61968,7 +61965,7 @@
         <v>925</v>
       </c>
       <c r="F43" s="64" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
       <c r="G43" s="38" t="s">
         <v>330</v>
@@ -61976,22 +61973,22 @@
     </row>
     <row r="44" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="64" t="s">
+        <v>1021</v>
+      </c>
+      <c r="B44" s="71" t="s">
         <v>1022</v>
       </c>
-      <c r="B44" s="71" t="s">
+      <c r="C44" s="13" t="s">
         <v>1023</v>
       </c>
-      <c r="C44" s="13" t="s">
+      <c r="D44" s="63" t="s">
         <v>1024</v>
       </c>
-      <c r="D44" s="63" t="s">
+      <c r="E44" s="63" t="s">
         <v>1025</v>
       </c>
-      <c r="E44" s="63" t="s">
+      <c r="F44" s="63" t="s">
         <v>1026</v>
-      </c>
-      <c r="F44" s="63" t="s">
-        <v>1027</v>
       </c>
       <c r="G44" s="41" t="s">
         <v>83</v>
@@ -62002,7 +61999,7 @@
     <hyperlink ref="B5" r:id="rId1" display="安敦國際大樓 ↗"/>
     <hyperlink ref="C5" r:id="rId2" display="https://business.591.com.tw/rent/22034644"/>
     <hyperlink ref="B6" r:id="rId3" display="安敦國際大樓 ↗"/>
-    <hyperlink ref="C6" r:id="rId4" display="https://www.sinyi.com.tw/rent/houseno/CZ05290"/>
+    <hyperlink ref="C6" r:id="rId4" display="https://www.sinyiglobal.com/rental/CZ05290"/>
     <hyperlink ref="B7" r:id="rId5" display="安敦國際大樓 ↗"/>
     <hyperlink ref="C7" r:id="rId6" display="https://www.sinyi.com.tw/communitylist/communityinfo/0008194"/>
     <hyperlink ref="B8" r:id="rId7" display="安敦國際大樓 ↗"/>
@@ -62040,7 +62037,7 @@
     <hyperlink ref="B26" r:id="rId39" display="白宮企業大樓 ↗"/>
     <hyperlink ref="C26" r:id="rId40" display="https://buy.housefun.com.tw/buy/building/28758"/>
     <hyperlink ref="B28" r:id="rId41" display="白宮企業大樓 — 同層參考(非本案) ↗"/>
-    <hyperlink ref="C28" r:id="rId42" display="https://www.sinyi.com.tw/rent/houseno/C351775"/>
+    <hyperlink ref="C28" r:id="rId42" display="https://www.sinyiglobal.com/rental/C351775"/>
     <hyperlink ref="B29" r:id="rId43" display="白宮企業大樓 — 同層參考(非本案) ↗"/>
     <hyperlink ref="C29" r:id="rId44" display="https://business.591.com.tw/rent/21646876"/>
     <hyperlink ref="B30" r:id="rId45" display="白宮企業大樓 — 同層參考(非本案) ↗"/>
@@ -62056,11 +62053,11 @@
     <hyperlink ref="B35" r:id="rId55" display="國泰建經 民生商業大樓 ↗"/>
     <hyperlink ref="C35" r:id="rId56" display="https://www.cathay-rem.com.tw/property/detail/743zt8ammFQReRwF"/>
     <hyperlink ref="B36" r:id="rId57" display="中鼎大樓 15F之1 ↗"/>
-    <hyperlink ref="C36" r:id="rId58" display="https://www.sinyi.com.tw/rent/houseno/CZ05572"/>
+    <hyperlink ref="C36" r:id="rId58" display="https://www.sinyiglobal.com/rental/CZ05572"/>
     <hyperlink ref="B37" r:id="rId59" display="中鼎大樓 2F ↗"/>
-    <hyperlink ref="C37" r:id="rId60" display="https://www.sinyi.com.tw/rent/houseno/CZ05228"/>
+    <hyperlink ref="C37" r:id="rId60" display="https://www.sinyiglobal.com/rental/CZ05228"/>
     <hyperlink ref="B38" r:id="rId61" display="家美金融大樓 15F ↗"/>
-    <hyperlink ref="C38" r:id="rId62" display="https://www.sinyi.com.tw/rent/houseno/CZ05491"/>
+    <hyperlink ref="C38" r:id="rId62" display="https://www.sinyiglobal.com/rental/CZ05491"/>
     <hyperlink ref="B39" r:id="rId63" display="永慶 安敦國際大樓 14F ↗"/>
     <hyperlink ref="C39" r:id="rId64" display="https://rent.yungching.com.tw/region/house/2358272?pc=0916263633"/>
     <hyperlink ref="B40" r:id="rId65" display="永慶 家美金融大樓 15F ↗"/>
@@ -62068,7 +62065,7 @@
     <hyperlink ref="B41" r:id="rId67" display="信義 光復北路新大樓 5F ↗"/>
     <hyperlink ref="C41" r:id="rId68" display="https://www.sinyiglobal.com/rental/C355686"/>
     <hyperlink ref="B42" r:id="rId69" display="信義 光復北路新大樓 5F ↗"/>
-    <hyperlink ref="C42" r:id="rId70" display="https://www.sinyi.com.tw/rent/houseno/C355686"/>
+    <hyperlink ref="C42" r:id="rId70" display="https://www.sinyiglobal.com/rental/C355686"/>
     <hyperlink ref="B43" r:id="rId71" display="鴻霖大樓 10F之2 ↗"/>
     <hyperlink ref="C43" r:id="rId72" display="https://kevinashowtimes-web.github.io/showtime-office-dashboard/JE_J07_honglin_10F-2.pdf"/>
     <hyperlink ref="B44" r:id="rId73" display="傑森愛華清單 ↗"/>
@@ -62104,12 +62101,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>1028</v>
+        <v>1027</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -62120,16 +62117,16 @@
         <v>3</v>
       </c>
       <c r="C4" s="68" t="s">
+        <v>1029</v>
+      </c>
+      <c r="D4" s="68" t="s">
         <v>1030</v>
       </c>
-      <c r="D4" s="68" t="s">
+      <c r="E4" s="68" t="s">
         <v>1031</v>
       </c>
-      <c r="E4" s="68" t="s">
+      <c r="F4" s="68" t="s">
         <v>1032</v>
-      </c>
-      <c r="F4" s="68" t="s">
-        <v>1033</v>
       </c>
       <c r="G4" s="68" t="s">
         <v>24</v>
@@ -62140,22 +62137,22 @@
     </row>
     <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="63" t="s">
-        <v>1034</v>
+        <v>1033</v>
       </c>
       <c r="B5" s="64" t="s">
         <v>323</v>
       </c>
       <c r="C5" s="63" t="s">
+        <v>1034</v>
+      </c>
+      <c r="D5" s="63" t="s">
         <v>1035</v>
       </c>
-      <c r="D5" s="63" t="s">
+      <c r="E5" s="63" t="s">
         <v>1036</v>
       </c>
-      <c r="E5" s="63" t="s">
+      <c r="F5" s="96" t="s">
         <v>1037</v>
-      </c>
-      <c r="F5" s="96" t="s">
-        <v>1038</v>
       </c>
       <c r="G5" s="25" t="s">
         <v>323</v>
@@ -62166,22 +62163,22 @@
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="63" t="s">
-        <v>1034</v>
+        <v>1033</v>
       </c>
       <c r="B6" s="64" t="s">
         <v>323</v>
       </c>
       <c r="C6" s="63" t="s">
+        <v>1038</v>
+      </c>
+      <c r="D6" s="63" t="s">
         <v>1039</v>
       </c>
-      <c r="D6" s="63" t="s">
-        <v>1040</v>
-      </c>
       <c r="E6" s="63" t="s">
+        <v>1036</v>
+      </c>
+      <c r="F6" s="96" t="s">
         <v>1037</v>
-      </c>
-      <c r="F6" s="96" t="s">
-        <v>1038</v>
       </c>
       <c r="G6" s="25" t="s">
         <v>323</v>
@@ -62192,22 +62189,22 @@
     </row>
     <row r="7" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="63" t="s">
-        <v>1034</v>
+        <v>1033</v>
       </c>
       <c r="B7" s="64" t="s">
         <v>323</v>
       </c>
       <c r="C7" s="63" t="s">
+        <v>1040</v>
+      </c>
+      <c r="D7" s="63" t="s">
         <v>1041</v>
       </c>
-      <c r="D7" s="63" t="s">
+      <c r="E7" s="63" t="s">
+        <v>1036</v>
+      </c>
+      <c r="F7" s="63" t="s">
         <v>1042</v>
-      </c>
-      <c r="E7" s="63" t="s">
-        <v>1037</v>
-      </c>
-      <c r="F7" s="63" t="s">
-        <v>1043</v>
       </c>
       <c r="G7" s="25" t="s">
         <v>323</v>
@@ -62224,16 +62221,16 @@
         <v>26</v>
       </c>
       <c r="C8" s="63" t="s">
+        <v>1043</v>
+      </c>
+      <c r="D8" s="63" t="s">
         <v>1044</v>
       </c>
-      <c r="D8" s="63" t="s">
+      <c r="E8" s="63" t="s">
         <v>1045</v>
       </c>
-      <c r="E8" s="63" t="s">
-        <v>1046</v>
-      </c>
       <c r="F8" s="96" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="G8" s="13" t="s">
         <v>37</v>
@@ -62250,16 +62247,16 @@
         <v>39</v>
       </c>
       <c r="C9" s="63" t="s">
+        <v>1046</v>
+      </c>
+      <c r="D9" s="63" t="s">
         <v>1047</v>
       </c>
-      <c r="D9" s="63" t="s">
+      <c r="E9" s="63" t="s">
         <v>1048</v>
       </c>
-      <c r="E9" s="63" t="s">
-        <v>1049</v>
-      </c>
       <c r="F9" s="96" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="G9" s="14" t="s">
         <v>48</v>
@@ -62276,16 +62273,16 @@
         <v>39</v>
       </c>
       <c r="C10" s="63" t="s">
+        <v>1049</v>
+      </c>
+      <c r="D10" s="63" t="s">
         <v>1050</v>
       </c>
-      <c r="D10" s="63" t="s">
-        <v>1051</v>
-      </c>
       <c r="E10" s="63" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
       <c r="F10" s="63" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
       <c r="G10" s="14" t="s">
         <v>48</v>
@@ -62302,16 +62299,16 @@
         <v>59</v>
       </c>
       <c r="C11" s="63" t="s">
+        <v>1051</v>
+      </c>
+      <c r="D11" s="63" t="s">
         <v>1052</v>
       </c>
-      <c r="D11" s="63" t="s">
+      <c r="E11" s="63" t="s">
         <v>1053</v>
       </c>
-      <c r="E11" s="63" t="s">
-        <v>1054</v>
-      </c>
       <c r="F11" s="96" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="G11" s="13" t="s">
         <v>68</v>
@@ -62328,16 +62325,16 @@
         <v>59</v>
       </c>
       <c r="C12" s="63" t="s">
+        <v>1054</v>
+      </c>
+      <c r="D12" s="63" t="s">
         <v>1055</v>
       </c>
-      <c r="D12" s="63" t="s">
-        <v>1056</v>
-      </c>
       <c r="E12" s="63" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
       <c r="F12" s="96" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="G12" s="13" t="s">
         <v>68</v>
@@ -62354,16 +62351,16 @@
         <v>70</v>
       </c>
       <c r="C13" s="63" t="s">
+        <v>1056</v>
+      </c>
+      <c r="D13" s="63" t="s">
         <v>1057</v>
       </c>
-      <c r="D13" s="63" t="s">
+      <c r="E13" s="63" t="s">
         <v>1058</v>
       </c>
-      <c r="E13" s="63" t="s">
-        <v>1059</v>
-      </c>
       <c r="F13" s="96" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="G13" s="14" t="s">
         <v>78</v>
@@ -62380,16 +62377,16 @@
         <v>70</v>
       </c>
       <c r="C14" s="63" t="s">
+        <v>1059</v>
+      </c>
+      <c r="D14" s="63" t="s">
         <v>1060</v>
       </c>
-      <c r="D14" s="63" t="s">
-        <v>1061</v>
-      </c>
       <c r="E14" s="63" t="s">
-        <v>1059</v>
+        <v>1058</v>
       </c>
       <c r="F14" s="96" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="G14" s="14" t="s">
         <v>78</v>
@@ -62406,16 +62403,16 @@
         <v>70</v>
       </c>
       <c r="C15" s="63" t="s">
+        <v>1061</v>
+      </c>
+      <c r="D15" s="63" t="s">
         <v>1062</v>
       </c>
-      <c r="D15" s="63" t="s">
-        <v>1063</v>
-      </c>
       <c r="E15" s="63" t="s">
-        <v>1059</v>
+        <v>1058</v>
       </c>
       <c r="F15" s="96" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="G15" s="14" t="s">
         <v>78</v>
@@ -62426,22 +62423,22 @@
     </row>
     <row r="16" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="64" t="s">
+        <v>1063</v>
+      </c>
+      <c r="B16" s="71" t="s">
         <v>1064</v>
       </c>
-      <c r="B16" s="71" t="s">
+      <c r="C16" s="63" t="s">
         <v>1065</v>
       </c>
-      <c r="C16" s="63" t="s">
+      <c r="D16" s="63" t="s">
         <v>1066</v>
       </c>
-      <c r="D16" s="63" t="s">
+      <c r="E16" s="63" t="s">
         <v>1067</v>
       </c>
-      <c r="E16" s="63" t="s">
-        <v>1068</v>
-      </c>
       <c r="F16" s="96" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="G16" s="14" t="s">
         <v>309</v>
@@ -62458,16 +62455,16 @@
         <v>80</v>
       </c>
       <c r="C17" s="63" t="s">
+        <v>1068</v>
+      </c>
+      <c r="D17" s="63" t="s">
         <v>1069</v>
       </c>
-      <c r="D17" s="63" t="s">
+      <c r="E17" s="63" t="s">
         <v>1070</v>
       </c>
-      <c r="E17" s="63" t="s">
-        <v>1071</v>
-      </c>
       <c r="F17" s="96" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="G17" s="14" t="s">
         <v>87</v>
@@ -62484,16 +62481,16 @@
         <v>80</v>
       </c>
       <c r="C18" s="63" t="s">
+        <v>1071</v>
+      </c>
+      <c r="D18" s="63" t="s">
         <v>1072</v>
       </c>
-      <c r="D18" s="63" t="s">
-        <v>1073</v>
-      </c>
       <c r="E18" s="63" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
       <c r="F18" s="63" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
       <c r="G18" s="14" t="s">
         <v>87</v>
@@ -62510,16 +62507,16 @@
         <v>80</v>
       </c>
       <c r="C19" s="63" t="s">
+        <v>1073</v>
+      </c>
+      <c r="D19" s="63" t="s">
         <v>1074</v>
       </c>
-      <c r="D19" s="63" t="s">
+      <c r="E19" s="63" t="s">
         <v>1075</v>
       </c>
-      <c r="E19" s="63" t="s">
-        <v>1076</v>
-      </c>
       <c r="F19" s="63" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
       <c r="G19" s="14" t="s">
         <v>87</v>
@@ -62536,16 +62533,16 @@
         <v>89</v>
       </c>
       <c r="C20" s="63" t="s">
+        <v>1076</v>
+      </c>
+      <c r="D20" s="63" t="s">
         <v>1077</v>
       </c>
-      <c r="D20" s="63" t="s">
-        <v>1078</v>
-      </c>
       <c r="E20" s="63" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
       <c r="F20" s="96" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="G20" s="14" t="s">
         <v>95</v>
@@ -62562,16 +62559,16 @@
         <v>89</v>
       </c>
       <c r="C21" s="63" t="s">
+        <v>1078</v>
+      </c>
+      <c r="D21" s="63" t="s">
         <v>1079</v>
       </c>
-      <c r="D21" s="63" t="s">
-        <v>1080</v>
-      </c>
       <c r="E21" s="63" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
       <c r="F21" s="96" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="G21" s="14" t="s">
         <v>95</v>
@@ -62588,16 +62585,16 @@
         <v>97</v>
       </c>
       <c r="C22" s="63" t="s">
+        <v>1080</v>
+      </c>
+      <c r="D22" s="63" t="s">
         <v>1081</v>
       </c>
-      <c r="D22" s="63" t="s">
+      <c r="E22" s="63" t="s">
         <v>1082</v>
       </c>
-      <c r="E22" s="63" t="s">
-        <v>1083</v>
-      </c>
       <c r="F22" s="96" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="G22" s="13" t="s">
         <v>104</v>
@@ -62614,16 +62611,16 @@
         <v>97</v>
       </c>
       <c r="C23" s="63" t="s">
+        <v>1083</v>
+      </c>
+      <c r="D23" s="64" t="s">
         <v>1084</v>
       </c>
-      <c r="D23" s="64" t="s">
+      <c r="E23" s="63" t="s">
         <v>1085</v>
       </c>
-      <c r="E23" s="63" t="s">
-        <v>1086</v>
-      </c>
       <c r="F23" s="96" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>104</v>
@@ -62640,16 +62637,16 @@
         <v>106</v>
       </c>
       <c r="C24" s="63" t="s">
+        <v>1086</v>
+      </c>
+      <c r="D24" s="63" t="s">
         <v>1087</v>
       </c>
-      <c r="D24" s="63" t="s">
+      <c r="E24" s="63" t="s">
         <v>1088</v>
       </c>
-      <c r="E24" s="63" t="s">
-        <v>1089</v>
-      </c>
       <c r="F24" s="96" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="G24" s="14" t="s">
         <v>114</v>
@@ -62666,16 +62663,16 @@
         <v>106</v>
       </c>
       <c r="C25" s="63" t="s">
+        <v>1089</v>
+      </c>
+      <c r="D25" s="63" t="s">
         <v>1090</v>
       </c>
-      <c r="D25" s="63" t="s">
+      <c r="E25" s="63" t="s">
         <v>1091</v>
       </c>
-      <c r="E25" s="63" t="s">
-        <v>1092</v>
-      </c>
       <c r="F25" s="96" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="G25" s="14" t="s">
         <v>114</v>
@@ -62692,16 +62689,16 @@
         <v>106</v>
       </c>
       <c r="C26" s="63" t="s">
+        <v>1092</v>
+      </c>
+      <c r="D26" s="63" t="s">
         <v>1093</v>
       </c>
-      <c r="D26" s="63" t="s">
+      <c r="E26" s="63" t="s">
         <v>1094</v>
       </c>
-      <c r="E26" s="63" t="s">
-        <v>1095</v>
-      </c>
       <c r="F26" s="96" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="G26" s="14" t="s">
         <v>114</v>
@@ -62712,22 +62709,22 @@
     </row>
     <row r="27" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="64" t="s">
+        <v>1095</v>
+      </c>
+      <c r="B27" s="72" t="s">
         <v>1096</v>
       </c>
-      <c r="B27" s="72" t="s">
+      <c r="C27" s="63" t="s">
         <v>1097</v>
       </c>
-      <c r="C27" s="63" t="s">
+      <c r="D27" s="63" t="s">
+        <v>1069</v>
+      </c>
+      <c r="E27" s="63" t="s">
         <v>1098</v>
       </c>
-      <c r="D27" s="63" t="s">
-        <v>1070</v>
-      </c>
-      <c r="E27" s="63" t="s">
-        <v>1099</v>
-      </c>
       <c r="F27" s="96" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="G27" s="13" t="s">
         <v>421</v>
@@ -62738,22 +62735,22 @@
     </row>
     <row r="28" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="64" t="s">
+        <v>1099</v>
+      </c>
+      <c r="B28" s="71" t="s">
         <v>1100</v>
       </c>
-      <c r="B28" s="71" t="s">
+      <c r="C28" s="63" t="s">
         <v>1101</v>
       </c>
-      <c r="C28" s="63" t="s">
+      <c r="D28" s="63" t="s">
         <v>1102</v>
       </c>
-      <c r="D28" s="63" t="s">
-        <v>1103</v>
-      </c>
       <c r="E28" s="63" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="F28" s="96" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="G28" s="14" t="s">
         <v>351</v>
@@ -62770,16 +62767,16 @@
         <v>39</v>
       </c>
       <c r="C29" s="63" t="s">
+        <v>1103</v>
+      </c>
+      <c r="D29" s="63" t="s">
         <v>1104</v>
       </c>
-      <c r="D29" s="63" t="s">
+      <c r="E29" s="63" t="s">
         <v>1105</v>
       </c>
-      <c r="E29" s="63" t="s">
-        <v>1106</v>
-      </c>
       <c r="F29" s="96" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="G29" s="14" t="s">
         <v>48</v>
@@ -62796,16 +62793,16 @@
         <v>59</v>
       </c>
       <c r="C30" s="63" t="s">
+        <v>1106</v>
+      </c>
+      <c r="D30" s="63" t="s">
         <v>1107</v>
       </c>
-      <c r="D30" s="63" t="s">
+      <c r="E30" s="63" t="s">
         <v>1108</v>
       </c>
-      <c r="E30" s="63" t="s">
-        <v>1109</v>
-      </c>
       <c r="F30" s="96" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="G30" s="13" t="s">
         <v>68</v>
@@ -62822,16 +62819,16 @@
         <v>59</v>
       </c>
       <c r="C31" s="64" t="s">
+        <v>1109</v>
+      </c>
+      <c r="D31" s="63" t="s">
         <v>1110</v>
       </c>
-      <c r="D31" s="63" t="s">
+      <c r="E31" s="63" t="s">
         <v>1111</v>
       </c>
-      <c r="E31" s="63" t="s">
-        <v>1112</v>
-      </c>
       <c r="F31" s="96" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>68</v>
@@ -62845,19 +62842,19 @@
         <v>323</v>
       </c>
       <c r="B32" s="63" t="s">
+        <v>1112</v>
+      </c>
+      <c r="C32" s="63" t="s">
         <v>1113</v>
       </c>
-      <c r="C32" s="63" t="s">
+      <c r="D32" s="63" t="s">
         <v>1114</v>
       </c>
-      <c r="D32" s="63" t="s">
+      <c r="E32" s="63" t="s">
         <v>1115</v>
       </c>
-      <c r="E32" s="63" t="s">
-        <v>1116</v>
-      </c>
       <c r="F32" s="63" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
       <c r="G32" s="25" t="s">
         <v>323</v>
@@ -62871,19 +62868,19 @@
         <v>157</v>
       </c>
       <c r="B33" s="71" t="s">
+        <v>1116</v>
+      </c>
+      <c r="C33" s="64" t="s">
         <v>1117</v>
-      </c>
-      <c r="C33" s="64" t="s">
-        <v>1118</v>
       </c>
       <c r="D33" s="63" t="s">
         <v>647</v>
       </c>
       <c r="E33" s="63" t="s">
-        <v>1119</v>
+        <v>1118</v>
       </c>
       <c r="F33" s="63" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
       <c r="G33" s="14" t="s">
         <v>167</v>
@@ -62897,19 +62894,19 @@
         <v>168</v>
       </c>
       <c r="B34" s="71" t="s">
+        <v>1119</v>
+      </c>
+      <c r="C34" s="63" t="s">
         <v>1120</v>
       </c>
-      <c r="C34" s="63" t="s">
+      <c r="D34" s="63" t="s">
         <v>1121</v>
       </c>
-      <c r="D34" s="63" t="s">
+      <c r="E34" s="63" t="s">
         <v>1122</v>
       </c>
-      <c r="E34" s="63" t="s">
-        <v>1123</v>
-      </c>
       <c r="F34" s="96" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="G34" s="14" t="s">
         <v>175</v>
@@ -62923,19 +62920,19 @@
         <v>147</v>
       </c>
       <c r="B35" s="71" t="s">
+        <v>1123</v>
+      </c>
+      <c r="C35" s="63" t="s">
         <v>1124</v>
       </c>
-      <c r="C35" s="63" t="s">
+      <c r="D35" s="63" t="s">
         <v>1125</v>
       </c>
-      <c r="D35" s="63" t="s">
+      <c r="E35" s="63" t="s">
         <v>1126</v>
       </c>
-      <c r="E35" s="63" t="s">
-        <v>1127</v>
-      </c>
       <c r="F35" s="63" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
       <c r="G35" s="14" t="s">
         <v>156</v>
@@ -62952,16 +62949,16 @@
         <v>116</v>
       </c>
       <c r="C36" s="64" t="s">
+        <v>1127</v>
+      </c>
+      <c r="D36" s="63" t="s">
         <v>1128</v>
       </c>
-      <c r="D36" s="63" t="s">
+      <c r="E36" s="63" t="s">
         <v>1129</v>
       </c>
-      <c r="E36" s="63" t="s">
-        <v>1130</v>
-      </c>
       <c r="F36" s="96" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="G36" s="14" t="s">
         <v>124</v>
@@ -62978,16 +62975,16 @@
         <v>1010</v>
       </c>
       <c r="C37" s="64" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D37" s="63" t="s">
         <v>1131</v>
       </c>
-      <c r="D37" s="63" t="s">
-        <v>1132</v>
-      </c>
       <c r="E37" s="63" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
       <c r="F37" s="96" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="G37" s="14" t="s">
         <v>136</v>
@@ -63001,19 +62998,19 @@
         <v>381</v>
       </c>
       <c r="B38" s="71" t="s">
+        <v>1132</v>
+      </c>
+      <c r="C38" s="63" t="s">
         <v>1133</v>
       </c>
-      <c r="C38" s="63" t="s">
+      <c r="D38" s="63" t="s">
         <v>1134</v>
       </c>
-      <c r="D38" s="63" t="s">
+      <c r="E38" s="63" t="s">
         <v>1135</v>
       </c>
-      <c r="E38" s="63" t="s">
-        <v>1136</v>
-      </c>
       <c r="F38" s="96" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="G38" s="14" t="s">
         <v>389</v>
@@ -63027,19 +63024,19 @@
         <v>381</v>
       </c>
       <c r="B39" s="71" t="s">
-        <v>1133</v>
+        <v>1132</v>
       </c>
       <c r="C39" s="63" t="s">
+        <v>1136</v>
+      </c>
+      <c r="D39" s="63" t="s">
         <v>1137</v>
       </c>
-      <c r="D39" s="63" t="s">
+      <c r="E39" s="63" t="s">
         <v>1138</v>
       </c>
-      <c r="E39" s="63" t="s">
-        <v>1139</v>
-      </c>
       <c r="F39" s="96" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="G39" s="14" t="s">
         <v>389</v>
@@ -63053,19 +63050,19 @@
         <v>381</v>
       </c>
       <c r="B40" s="71" t="s">
-        <v>1133</v>
+        <v>1132</v>
       </c>
       <c r="C40" s="63" t="s">
+        <v>1139</v>
+      </c>
+      <c r="D40" s="63" t="s">
         <v>1140</v>
       </c>
-      <c r="D40" s="63" t="s">
-        <v>1141</v>
-      </c>
       <c r="E40" s="63" t="s">
-        <v>1139</v>
+        <v>1138</v>
       </c>
       <c r="F40" s="63" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
       <c r="G40" s="14" t="s">
         <v>389</v>
@@ -63079,19 +63076,19 @@
         <v>493</v>
       </c>
       <c r="B41" s="71" t="s">
+        <v>1141</v>
+      </c>
+      <c r="C41" s="63" t="s">
         <v>1142</v>
       </c>
-      <c r="C41" s="63" t="s">
+      <c r="D41" s="63" t="s">
         <v>1143</v>
       </c>
-      <c r="D41" s="63" t="s">
+      <c r="E41" s="63" t="s">
         <v>1144</v>
       </c>
-      <c r="E41" s="63" t="s">
-        <v>1145</v>
-      </c>
       <c r="F41" s="63" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
       <c r="G41" s="14" t="s">
         <v>499</v>
@@ -63105,19 +63102,19 @@
         <v>474</v>
       </c>
       <c r="B42" s="71" t="s">
+        <v>1145</v>
+      </c>
+      <c r="C42" s="63" t="s">
         <v>1146</v>
       </c>
-      <c r="C42" s="63" t="s">
+      <c r="D42" s="64" t="s">
         <v>1147</v>
       </c>
-      <c r="D42" s="64" t="s">
-        <v>1148</v>
-      </c>
       <c r="E42" s="63" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="F42" s="63" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
       <c r="G42" s="14" t="s">
         <v>480</v>
@@ -63161,11 +63158,11 @@
     <hyperlink ref="B23" r:id="rId31" display="591 光復南路 7F ↗"/>
     <hyperlink ref="G23" r:id="rId32" display="HouseWeb 本戶·40張照片"/>
     <hyperlink ref="B24" r:id="rId33" display="信義 光復北路新大樓 5F ↗"/>
-    <hyperlink ref="G24" r:id="rId34" display="信義國際站 本戶·14張照片（備用：www.sinyi.com.tw/rent/houseno/C355686）"/>
+    <hyperlink ref="G24" r:id="rId34" display="信義全球 本戶·14張照片（C355686）"/>
     <hyperlink ref="B25" r:id="rId35" display="信義 光復北路新大樓 5F ↗"/>
-    <hyperlink ref="G25" r:id="rId36" display="信義國際站 本戶·14張照片（備用：www.sinyi.com.tw/rent/houseno/C355686）"/>
+    <hyperlink ref="G25" r:id="rId36" display="信義全球 本戶·14張照片（C355686）"/>
     <hyperlink ref="B26" r:id="rId37" display="信義 光復北路新大樓 5F ↗"/>
-    <hyperlink ref="G26" r:id="rId38" display="信義國際站 本戶·14張照片（備用：www.sinyi.com.tw/rent/houseno/C355686）"/>
+    <hyperlink ref="G26" r:id="rId38" display="信義全球 本戶·14張照片（C355686）"/>
     <hyperlink ref="B27" r:id="rId39" display="HouseWeb 兩案 ↗"/>
     <hyperlink ref="G27" r:id="rId40" display="HouseWeb·38張"/>
     <hyperlink ref="B28" r:id="rId41" location="page=1" display="傑森愛華全部(&lt;200坪已刪) ↗"/>

</xml_diff>